<commit_message>
Sod, approver, deployer all were tested
</commit_message>
<xml_diff>
--- a/src/data/output/sod_violations/sod_violations.xlsx
+++ b/src/data/output/sod_violations/sod_violations.xlsx
@@ -544,14 +544,10 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Exception</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Requestor and Approver share the same ID (USR001)</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -978,14 +974,10 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Exception</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Requestor and Approver share the same ID (USR008)</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1102,14 +1094,10 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Exception</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Requestor and Approver share the same ID (USR010)</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1164,10 +1152,14 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
+          <t>Exception</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Requestor and Approver share the same ID (USR011)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1222,10 +1214,14 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
+          <t>Exception</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Requestor and Approver share the same ID (USR011)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1280,10 +1276,14 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
+          <t>Exception</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Requestor and Approver share the same ID (USR012)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1338,10 +1338,14 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
+          <t>Exception</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Requestor and Approver share the same ID (USR013)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1396,10 +1400,14 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
+          <t>Exception</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Requestor and Approver share the same ID (USR014)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2357,7 +2365,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Deployer and Approver share the same ID (USR030)</t>
+          <t>Approver and Deployer share the same ID (USR030)</t>
         </is>
       </c>
     </row>
@@ -2395,7 +2403,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025-12-10 18:40:55</t>
+          <t>2026-02-04 11:40:39</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2448,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">

</xml_diff>